<commit_message>
Ưu tiên TrangThai/GhiChu từ kết quả import khi ghi sheet kiểm tra
Co-authored-by: thaison20101 <thaison20101@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kskdk-tthc-nhap-lieu/KSKDK_TTHC_mau_nhap_c2cd_kiem_tra.xlsx
+++ b/kskdk-tthc-nhap-lieu/KSKDK_TTHC_mau_nhap_c2cd_kiem_tra.xlsx
@@ -677,6 +677,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>082185000807</t>
@@ -697,6 +698,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>0937721349</t>
@@ -717,14 +722,27 @@
           <t>Phường Bình Tân</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA2" t="n">
@@ -757,6 +775,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>079300009617</t>
@@ -777,6 +796,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>0708731758</t>
@@ -797,14 +820,27 @@
           <t>Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA3" t="n">
@@ -837,6 +873,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>080185001753</t>
@@ -857,6 +894,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
           <t>0933854046</t>
@@ -877,14 +918,27 @@
           <t xml:space="preserve"> Phường Phú Định</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA4" t="n">
@@ -917,6 +971,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>079185000629</t>
@@ -937,6 +992,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
           <t>0989879633</t>
@@ -957,14 +1016,27 @@
           <t xml:space="preserve"> Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA5" t="n">
@@ -997,6 +1069,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>079188037353</t>
@@ -1017,6 +1090,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
           <t>0908202205</t>
@@ -1037,14 +1114,27 @@
           <t xml:space="preserve"> Phường Bình Đông </t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA6" t="n">
@@ -1077,6 +1167,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>079179025392</t>
@@ -1097,6 +1188,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
           <t>0907227307</t>
@@ -1117,14 +1212,27 @@
           <t xml:space="preserve"> Phường Tân Phú</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA7" t="n">
@@ -1157,6 +1265,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>079185025540</t>
@@ -1177,6 +1286,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>0937333328</t>
@@ -1197,14 +1310,27 @@
           <t xml:space="preserve"> Phường Bình Hưng Hoà </t>
         </is>
       </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA8" t="n">
@@ -1237,6 +1363,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>079174031765</t>
@@ -1257,6 +1384,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>0918632174</t>
@@ -1277,14 +1408,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA9" t="n">
@@ -1317,6 +1461,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>051190000049</t>
@@ -1337,6 +1482,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>0357202138</t>
@@ -1357,14 +1506,27 @@
           <t xml:space="preserve"> Phường Tân Phú</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA10" t="n">
@@ -1397,6 +1559,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>054185005288</t>
@@ -1417,6 +1580,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>0867460909</t>
@@ -1437,14 +1604,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA11" t="n">
@@ -1477,6 +1657,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>075183016701</t>
@@ -1497,6 +1678,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
           <t>0903011541</t>
@@ -1517,14 +1702,27 @@
           <t xml:space="preserve"> Phường Phú Thạnh</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA12" t="n">
@@ -1557,6 +1755,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>083181005221</t>
@@ -1577,6 +1776,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
           <t>0908645695</t>
@@ -1597,14 +1800,27 @@
           <t xml:space="preserve"> Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA13" t="n">
@@ -1637,6 +1853,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>082185000807</t>
@@ -1657,6 +1874,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
           <t>0937721349</t>
@@ -1677,14 +1898,27 @@
           <t xml:space="preserve"> Phường Bình Tân</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA14" t="n">
@@ -1717,6 +1951,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>079188009614</t>
@@ -1737,6 +1972,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>0933128839</t>
@@ -1757,14 +1996,27 @@
           <t xml:space="preserve"> Phường Tân Phú </t>
         </is>
       </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA15" t="n">
@@ -1797,6 +2049,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>079182011955</t>
@@ -1817,6 +2070,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>0909960226</t>
@@ -1837,14 +2094,27 @@
           <t xml:space="preserve"> Phường Hòa Bình</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA16" t="n">
@@ -1877,6 +2147,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>040193011868</t>
@@ -1897,6 +2168,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>0986765546</t>
@@ -1917,14 +2192,27 @@
           <t xml:space="preserve"> Phường Bình Phú</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 28/07/2026</t>
         </is>
       </c>
       <c r="AA17" t="n">
@@ -1957,6 +2245,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>079300009617</t>
@@ -1977,6 +2266,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
           <t>0708731758</t>
@@ -1997,14 +2290,27 @@
           <t xml:space="preserve"> Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA18" t="n">
@@ -2037,6 +2343,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>007917603006</t>
@@ -2057,6 +2364,10 @@
           <t xml:space="preserve">Nữ </t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>0938579546</t>
@@ -2077,14 +2388,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Mã định danh không đúng định dạng hoặc không khớp với ngày sinh/giới tính!</t>
         </is>
       </c>
       <c r="AA19" t="n">
@@ -2117,6 +2441,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>083188003692</t>
@@ -2137,6 +2462,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>0976143923</t>
@@ -2157,14 +2486,27 @@
           <t xml:space="preserve"> Phường Bình Đông</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA20" t="n">
@@ -2197,6 +2539,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>087187000236</t>
@@ -2217,6 +2560,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>0989681925</t>
@@ -2237,14 +2584,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA21" t="n">
@@ -2277,6 +2637,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>060191000141</t>
@@ -2297,6 +2658,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
           <t>0703355736</t>
@@ -2317,14 +2682,27 @@
           <t xml:space="preserve"> Phường Bình Trị Đông</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA22" t="n">
@@ -2357,6 +2735,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>075199000029</t>
@@ -2377,6 +2756,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>0907192870</t>
@@ -2397,14 +2780,27 @@
           <t xml:space="preserve"> Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA23" t="n">
@@ -2437,6 +2833,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>068180000030</t>
@@ -2457,6 +2854,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>0909700300</t>
@@ -2477,14 +2878,27 @@
           <t xml:space="preserve"> Phường Phú Trung</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>DiaChiHienTai_XaPhuong: không map được ' Phường Phú Trung' — thử xem GoiY_XaPhuong. (KeyError("Không map được giá trị ' Phường Phú Trung'"))</t>
         </is>
       </c>
       <c r="AA24" t="n">
@@ -2517,6 +2931,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>092193002768</t>
@@ -2537,6 +2952,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>0936864894</t>
@@ -2557,14 +2976,27 @@
           <t>Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA25" t="n">
@@ -2597,6 +3029,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>080174008274</t>
@@ -2617,6 +3050,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>0392410909</t>
@@ -2637,14 +3074,27 @@
           <t xml:space="preserve">  Phường Phú Thọ</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA26" t="n">
@@ -2677,6 +3127,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>079175028956</t>
@@ -2697,6 +3148,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>0937220112</t>
@@ -2717,14 +3172,27 @@
           <t xml:space="preserve"> Phường Bình Đông</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA27" t="n">
@@ -2757,6 +3225,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>079168016119</t>
@@ -2777,6 +3246,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
           <t>0833301266</t>
@@ -2797,14 +3270,27 @@
           <t xml:space="preserve"> Phường Chợ Quán</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA28" t="n">
@@ -2837,6 +3323,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>079092008279</t>
@@ -2857,6 +3344,10 @@
           <t>Nam</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
           <t>0909542931</t>
@@ -2877,14 +3368,27 @@
           <t xml:space="preserve"> Xã Bình Hưng</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
           <t>Người chăm sóc, bảo vệ tòa nhà</t>
         </is>
       </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA29" t="n">
@@ -3097,6 +3601,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>082185000807</t>
@@ -3117,6 +3622,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>0937721349</t>
@@ -3137,14 +3646,27 @@
           <t>Phường Bình Tân</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA2" t="n">
@@ -3177,6 +3699,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>079300009617</t>
@@ -3197,6 +3720,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>0708731758</t>
@@ -3217,14 +3744,27 @@
           <t>Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA3" t="n">
@@ -3257,6 +3797,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>080185001753</t>
@@ -3277,6 +3818,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
           <t>0933854046</t>
@@ -3297,14 +3842,27 @@
           <t xml:space="preserve"> Phường Phú Định</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA4" t="n">
@@ -3337,6 +3895,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>079185000629</t>
@@ -3357,6 +3916,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
           <t>0989879633</t>
@@ -3377,14 +3940,27 @@
           <t xml:space="preserve"> Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA5" t="n">
@@ -3417,6 +3993,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>079188037353</t>
@@ -3437,6 +4014,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
           <t>0908202205</t>
@@ -3457,14 +4038,27 @@
           <t xml:space="preserve"> Phường Bình Đông </t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA6" t="n">
@@ -3497,6 +4091,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>079179025392</t>
@@ -3517,6 +4112,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
           <t>0907227307</t>
@@ -3537,14 +4136,27 @@
           <t xml:space="preserve"> Phường Tân Phú</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA7" t="n">
@@ -3577,6 +4189,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>079185025540</t>
@@ -3597,6 +4210,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>0937333328</t>
@@ -3617,14 +4234,27 @@
           <t xml:space="preserve"> Phường Bình Hưng Hoà </t>
         </is>
       </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA8" t="n">
@@ -3657,6 +4287,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>079174031765</t>
@@ -3677,6 +4308,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>0918632174</t>
@@ -3697,14 +4332,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA9" t="n">
@@ -3737,6 +4385,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>051190000049</t>
@@ -3757,6 +4406,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>0357202138</t>
@@ -3777,14 +4430,27 @@
           <t xml:space="preserve"> Phường Tân Phú</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA10" t="n">
@@ -3817,6 +4483,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>054185005288</t>
@@ -3837,6 +4504,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>0867460909</t>
@@ -3857,14 +4528,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA11" t="n">
@@ -3897,6 +4581,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>075183016701</t>
@@ -3917,6 +4602,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
           <t>0903011541</t>
@@ -3937,14 +4626,27 @@
           <t xml:space="preserve"> Phường Phú Thạnh</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA12" t="n">
@@ -3977,6 +4679,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>083181005221</t>
@@ -3997,6 +4700,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
           <t>0908645695</t>
@@ -4017,14 +4724,27 @@
           <t xml:space="preserve"> Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA13" t="n">
@@ -4057,6 +4777,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>082185000807</t>
@@ -4077,6 +4798,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
           <t>0937721349</t>
@@ -4097,14 +4822,27 @@
           <t xml:space="preserve"> Phường Bình Tân</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA14" t="n">
@@ -4137,6 +4875,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>079188009614</t>
@@ -4157,6 +4896,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>0933128839</t>
@@ -4177,14 +4920,27 @@
           <t xml:space="preserve"> Phường Tân Phú </t>
         </is>
       </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA15" t="n">
@@ -4217,6 +4973,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>079182011955</t>
@@ -4237,6 +4994,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>0909960226</t>
@@ -4257,14 +5018,27 @@
           <t xml:space="preserve"> Phường Hòa Bình</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA16" t="n">
@@ -4297,6 +5071,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>040193011868</t>
@@ -4317,6 +5092,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>0986765546</t>
@@ -4337,14 +5116,27 @@
           <t xml:space="preserve"> Phường Bình Phú</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 28/07/2026</t>
         </is>
       </c>
       <c r="AA17" t="n">
@@ -4377,6 +5169,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>079300009617</t>
@@ -4397,6 +5190,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
           <t>0708731758</t>
@@ -4417,14 +5214,27 @@
           <t xml:space="preserve"> Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA18" t="n">
@@ -4457,6 +5267,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>083188003692</t>
@@ -4477,6 +5288,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>0976143923</t>
@@ -4497,14 +5312,27 @@
           <t xml:space="preserve"> Phường Bình Đông</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA19" t="n">
@@ -4537,6 +5365,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>087187000236</t>
@@ -4557,6 +5386,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>0989681925</t>
@@ -4577,14 +5410,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 29/07/2026</t>
         </is>
       </c>
       <c r="AA20" t="n">
@@ -4617,6 +5463,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>060191000141</t>
@@ -4637,6 +5484,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>0703355736</t>
@@ -4657,14 +5508,27 @@
           <t xml:space="preserve"> Phường Bình Trị Đông</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA21" t="n">
@@ -4697,6 +5561,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>075199000029</t>
@@ -4717,6 +5582,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
           <t>0907192870</t>
@@ -4737,14 +5606,27 @@
           <t xml:space="preserve"> Phường Bình Tây</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA22" t="n">
@@ -4777,6 +5659,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>092193002768</t>
@@ -4797,6 +5680,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>0936864894</t>
@@ -4817,14 +5704,27 @@
           <t>Phường Minh Phụng</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA23" t="n">
@@ -4857,6 +5757,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>080174008274</t>
@@ -4877,6 +5778,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>0392410909</t>
@@ -4897,14 +5802,27 @@
           <t xml:space="preserve">  Phường Phú Thọ</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA24" t="n">
@@ -4937,6 +5855,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>079175028956</t>
@@ -4957,6 +5876,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>0937220112</t>
@@ -4977,14 +5900,27 @@
           <t xml:space="preserve"> Phường Bình Đông</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA25" t="n">
@@ -5017,6 +5953,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>079168016119</t>
@@ -5037,6 +5974,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>0833301266</t>
@@ -5057,14 +5998,27 @@
           <t xml:space="preserve"> Phường Chợ Quán</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
           <t>Nhân viên phục vụ đồ ăn uống</t>
         </is>
       </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA26" t="n">
@@ -5097,6 +6051,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>079092008279</t>
@@ -5117,6 +6072,10 @@
           <t>Nam</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>0909542931</t>
@@ -5137,14 +6096,27 @@
           <t xml:space="preserve"> Xã Bình Hưng</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
           <t>Người chăm sóc, bảo vệ tòa nhà</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>TRUNG</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>Công dân đã khám bằng 'Ngân sách nhà nước' tại Phòng khám đa khoa (thuộc Công ty TNHH Phòng khám đa khoa Thuận Kiều) vào ngày 23/07/2026</t>
         </is>
       </c>
       <c r="AA27" t="n">
@@ -5357,6 +6329,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>007917603006</t>
@@ -5377,6 +6350,10 @@
           <t xml:space="preserve">Nữ </t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>0938579546</t>
@@ -5397,14 +6374,27 @@
           <t xml:space="preserve"> Phường Bình Thới</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Mã định danh không đúng định dạng hoặc không khớp với ngày sinh/giới tính!</t>
         </is>
       </c>
       <c r="AA2" t="n">
@@ -5437,6 +6427,7 @@
           <t>Khám Theo Hợp Đồng</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>068180000030</t>
@@ -5457,6 +6448,10 @@
           <t>Nữ</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>0909700300</t>
@@ -5477,14 +6472,27 @@
           <t xml:space="preserve"> Phường Phú Trung</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>GIÁO VIÊN MẦM NON</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
           <t>Khám sức khỏe định kỳ</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>DiaChiHienTai_XaPhuong: không map được ' Phường Phú Trung' — thử xem GoiY_XaPhuong. (KeyError("Không map được giá trị ' Phường Phú Trung'"))</t>
         </is>
       </c>
       <c r="AA3" t="n">

</xml_diff>